<commit_message>
Sync Meat and Fish schedule for 2026-10-04
</commit_message>
<xml_diff>
--- a/График_подготовки_Зимний фестиваль _Мясо-Рыба.xlsx
+++ b/График_подготовки_Зимний фестиваль _Мясо-Рыба.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kakorolkova\Desktop\Новая папка\Заполнено_в работу\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kakorolkova\Nextcloud\Проекты\Королькова\Мясо-Рыба\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F9EBD76-FC8F-4C22-8E63-FEE3C9C86B30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCB7EF0B-48EA-4E46-B570-97F282545B35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="График" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="60">
   <si>
     <t xml:space="preserve">Первый этап: 25 декабря 2026 — 1 января 2027
 Перерыв: 2–3 января
@@ -198,6 +198,12 @@
   </si>
   <si>
     <t>Разработать детальную программу мероприятий подходящую по тематике</t>
+  </si>
+  <si>
+    <t>29.09.26 предварительно подготовлен</t>
+  </si>
+  <si>
+    <t>предварительно расчет 3000 за каждые 7 дней</t>
   </si>
 </sst>
 </file>
@@ -340,7 +346,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -406,25 +412,22 @@
     <xf numFmtId="14" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -647,21 +650,21 @@
     <col min="1" max="1" width="6.33203125" style="12" customWidth="1"/>
     <col min="2" max="2" width="53.4140625" style="8" customWidth="1"/>
     <col min="3" max="4" width="13" style="17" customWidth="1"/>
-    <col min="5" max="5" width="23.9140625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="27.5" style="2" customWidth="1"/>
     <col min="6" max="6" width="8.6640625" style="2"/>
-    <col min="7" max="7" width="16.33203125" style="29" customWidth="1"/>
+    <col min="7" max="7" width="16.33203125" style="25" customWidth="1"/>
     <col min="8" max="16384" width="8.6640625" style="2"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:7" ht="67.5" customHeight="1">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="26" t="s">
         <v>53</v>
       </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="25"/>
-      <c r="G2" s="28" t="s">
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="28"/>
+      <c r="G2" s="24" t="s">
         <v>0</v>
       </c>
     </row>
@@ -696,13 +699,15 @@
       <c r="B5" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="C5" s="26">
+      <c r="C5" s="16">
         <v>46337</v>
       </c>
-      <c r="D5" s="26">
+      <c r="D5" s="16">
         <v>46339</v>
       </c>
-      <c r="E5" s="1"/>
+      <c r="E5" s="7" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="6" spans="1:7" ht="36.5" customHeight="1">
       <c r="A6" s="10">
@@ -711,10 +716,10 @@
       <c r="B6" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="26">
+      <c r="C6" s="16">
         <v>46337</v>
       </c>
-      <c r="D6" s="26">
+      <c r="D6" s="16">
         <v>46343</v>
       </c>
       <c r="E6" s="1"/>
@@ -726,10 +731,10 @@
       <c r="B7" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="C7" s="26">
+      <c r="C7" s="16">
         <v>46337</v>
       </c>
-      <c r="D7" s="26">
+      <c r="D7" s="16">
         <v>46343</v>
       </c>
       <c r="E7" s="1"/>
@@ -741,10 +746,10 @@
       <c r="B8" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="26">
+      <c r="C8" s="16">
         <v>46337</v>
       </c>
-      <c r="D8" s="26">
+      <c r="D8" s="16">
         <v>46343</v>
       </c>
       <c r="E8" s="1"/>
@@ -756,10 +761,10 @@
       <c r="B9" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="C9" s="26">
+      <c r="C9" s="16">
         <v>46337</v>
       </c>
-      <c r="D9" s="26">
+      <c r="D9" s="16">
         <v>46343</v>
       </c>
       <c r="E9" s="7" t="s">
@@ -773,10 +778,10 @@
       <c r="B10" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="26">
+      <c r="C10" s="16">
         <v>46337</v>
       </c>
-      <c r="D10" s="26">
+      <c r="D10" s="16">
         <v>46343</v>
       </c>
       <c r="E10" s="1"/>
@@ -788,10 +793,10 @@
       <c r="B11" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="26">
+      <c r="C11" s="16">
         <v>46343</v>
       </c>
-      <c r="D11" s="26">
+      <c r="D11" s="16">
         <v>46356</v>
       </c>
       <c r="E11" s="1"/>
@@ -803,10 +808,10 @@
       <c r="B12" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="C12" s="26">
+      <c r="C12" s="16">
         <v>46359</v>
       </c>
-      <c r="D12" s="26">
+      <c r="D12" s="16">
         <v>46373</v>
       </c>
       <c r="E12" s="1"/>
@@ -818,58 +823,64 @@
       <c r="B13" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="27">
+      <c r="C13" s="23">
         <v>46337</v>
       </c>
-      <c r="D13" s="27">
+      <c r="D13" s="23">
         <v>46353</v>
       </c>
       <c r="E13" s="1"/>
     </row>
-    <row r="14" spans="1:7" ht="20" customHeight="1">
+    <row r="14" spans="1:7" ht="28.5" customHeight="1">
       <c r="A14" s="11" t="s">
         <v>12</v>
       </c>
       <c r="B14" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="C14" s="26">
+      <c r="C14" s="16">
         <v>46337</v>
       </c>
-      <c r="D14" s="26">
+      <c r="D14" s="16">
         <v>46344</v>
       </c>
-      <c r="E14" s="1"/>
-    </row>
-    <row r="15" spans="1:7" ht="20" customHeight="1">
+      <c r="E14" s="7" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="28.5" customHeight="1">
       <c r="A15" s="10" t="s">
         <v>14</v>
       </c>
       <c r="B15" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="C15" s="26">
+      <c r="C15" s="16">
         <v>46343</v>
       </c>
-      <c r="D15" s="26">
+      <c r="D15" s="16">
         <v>46344</v>
       </c>
-      <c r="E15" s="1"/>
-    </row>
-    <row r="16" spans="1:7" ht="20" customHeight="1">
+      <c r="E15" s="7" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="34" customHeight="1">
       <c r="A16" s="11" t="s">
         <v>16</v>
       </c>
       <c r="B16" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="C16" s="26">
+      <c r="C16" s="16">
         <v>46339</v>
       </c>
-      <c r="D16" s="26">
+      <c r="D16" s="16">
         <v>46352</v>
       </c>
-      <c r="E16" s="1"/>
+      <c r="E16" s="7" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="17" spans="1:5" ht="20" customHeight="1">
       <c r="A17" s="10">

</xml_diff>